<commit_message>
Fix import quality: header removal, section breaks, FAQ dedup, tracking pixels
- Fix cleanup transformer: use bare 'header' selector instead of 'header#mainHeader'
  (the id was on a child div, not the header tag itself)
- Add tracking pixel removal for analytics images (DoubleClick, Bing, Twitter, etc.)
- Move section boundary detection before parsers run in import script
  (section selectors use :has() on elements that parsers replace)
- Remove etrade-sections transformer from pipeline (logic now inline)
- Fix accordion-faq parser to deduplicate collapsed/expanded state entries
- Re-import all 6 pages with improved quality

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-product-detail-page.report.xlsx
+++ b/tools/importer/reports/import-product-detail-page.report.xlsx
@@ -52,7 +52,7 @@
     <t>product-detail-page</t>
   </si>
   <si>
-    <t>2026-03-19T20:51:40.995Z</t>
+    <t>2026-03-20T14:47:48.161Z</t>
   </si>
   <si>
     <t>Online Banking: Savings, Checking, CDs | Morgan Stanley Private Bank</t>
@@ -70,7 +70,7 @@
     <t>bank/certificate-of-deposit</t>
   </si>
   <si>
-    <t>2026-03-19T20:52:06.932Z</t>
+    <t>2026-03-20T14:48:11.741Z</t>
   </si>
   <si>
     <t>Certificate of Deposit | Compare CD Rates | E*TRADE</t>
@@ -85,7 +85,7 @@
     <t>bank/checking</t>
   </si>
   <si>
-    <t>2026-03-19T20:52:00.834Z</t>
+    <t>2026-03-20T14:48:05.657Z</t>
   </si>
   <si>
     <t>E*TRADE Checking Account: $0 Fee Online Banking</t>
@@ -103,7 +103,7 @@
     <t>bank/line-of-credit</t>
   </si>
   <si>
-    <t>2026-03-19T20:52:14.889Z</t>
+    <t>2026-03-20T14:48:18.414Z</t>
   </si>
   <si>
     <t>Agreement Library | E*TRADE</t>
@@ -121,7 +121,7 @@
     <t>bank/max-rate-checking</t>
   </si>
   <si>
-    <t>2026-03-19T20:51:54.290Z</t>
+    <t>2026-03-20T14:47:59.539Z</t>
   </si>
   <si>
     <t>Max-Rate Checking: High-Yield Checking Account | E*TRADE</t>
@@ -139,7 +139,7 @@
     <t>bank/premium-savings-account</t>
   </si>
   <si>
-    <t>2026-03-19T20:51:47.513Z</t>
+    <t>2026-03-20T14:47:53.098Z</t>
   </si>
   <si>
     <t>Premium Savings Account: 3.75% APY For 6 Months | E*TRADE</t>

</xml_diff>